<commit_message>
Add SQL Analytics, Advanced SQL, and Business Case Studies
</commit_message>
<xml_diff>
--- a/01_Data_Engineering/06_excel_analysis/02_data_validation.xlsx
+++ b/01_Data_Engineering/06_excel_analysis/02_data_validation.xlsx
@@ -8,13 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ANTO ABRAHAM AJ\Downloads\Enterprise_FinTech_Payment_Intelligence_Platform\01_Data_Engineering\06_excel_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7135D270-15EA-450D-A3F4-30ACF2F14F77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FBCFC37B-76BF-4133-A9E0-2B3ADA9A5CD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{52E292D0-837B-49FA-89D2-D88BFD2E4709}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{814779D7-9443-46E9-A9F7-4457F04ACA21}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Validation Summary" sheetId="1" r:id="rId1"/>
+    <sheet name="Fraud Validation" sheetId="2" r:id="rId2"/>
+    <sheet name="Referential Integrity" sheetId="3" r:id="rId3"/>
+    <sheet name="Financial Validation" sheetId="4" r:id="rId4"/>
+    <sheet name="Executive Summary" sheetId="5" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Validation Summary'!$A$1:$D$10</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,37 +46,273 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="8">
-  <si>
-    <t>Validation Rule</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="47">
+  <si>
+    <t>Validation Check</t>
+  </si>
+  <si>
+    <t>Expected Result</t>
+  </si>
+  <si>
+    <t>Actual Result</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Total Transactions Loaded</t>
+  </si>
+  <si>
+    <t>✅ PASS</t>
+  </si>
+  <si>
+    <t>Orphaned Time Keys</t>
+  </si>
+  <si>
+    <t>Orphaned Transaction Types</t>
+  </si>
+  <si>
+    <t>Orphaned Fraud Keys</t>
+  </si>
+  <si>
+    <t>Orphaned Source Accounts</t>
+  </si>
+  <si>
+    <t>Orphaned Destination Accounts</t>
+  </si>
+  <si>
+    <t>Negative Transaction Amounts</t>
+  </si>
+  <si>
+    <t>NULL Financial Values</t>
+  </si>
+  <si>
+    <t>Duplicate Transaction IDs</t>
+  </si>
+  <si>
+    <t>IsFraud</t>
+  </si>
+  <si>
+    <t>IsFlaggedFraud</t>
+  </si>
+  <si>
+    <t>Transactions</t>
+  </si>
+  <si>
+    <t>Dimension</t>
+  </si>
+  <si>
+    <t>Orphan Records</t>
+  </si>
+  <si>
+    <t>Dim_Time</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>Dim_TransactionType</t>
+  </si>
+  <si>
+    <t>Dim_Fraud</t>
+  </si>
+  <si>
+    <t>Dim_SourceAccount</t>
+  </si>
+  <si>
+    <t>Dim_DestinationAccount</t>
+  </si>
+  <si>
+    <t>Check</t>
   </si>
   <si>
     <t>Result</t>
   </si>
   <si>
-    <t>NULL Values</t>
+    <t>Negative Amounts</t>
+  </si>
+  <si>
+    <t>NULL Amount</t>
+  </si>
+  <si>
+    <t>NULL OldBalanceOrig</t>
+  </si>
+  <si>
+    <t>NULL NewBalanceOrig</t>
+  </si>
+  <si>
+    <t>NULL OldBalanceDest</t>
+  </si>
+  <si>
+    <t>NULL NewBalanceDest</t>
+  </si>
+  <si>
+    <t>Validation Statistics</t>
+  </si>
+  <si>
+    <t>Metric</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Total Transactions</t>
+  </si>
+  <si>
+    <t>Validation Checks</t>
   </si>
   <si>
     <t>Passed</t>
   </si>
   <si>
-    <t>Duplicate Records</t>
-  </si>
-  <si>
-    <t>Negative Amount</t>
-  </si>
-  <si>
-    <t>Invalid Transaction Type</t>
-  </si>
-  <si>
-    <t>Foreign Key Validation</t>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>Overall Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                 PASS</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Key Findings</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+1.All transaction records loaded successfully into the warehouse.
+2.No referential integrity violations were detected.
+3.Financial measures contain no invalid or missing values.
+4.Fraud labels were loaded correctly into the star schema.
+5.The warehouse is production-ready for analytics and reporting.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Financial Quality Assessment</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+1.No invalid financial values were detected.
+2.All transaction measures satisfy business validation rules.
+3.The fact table is suitable for analytical reporting.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Conclusion:  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">             1. All foreign key relationships are valid.
+2.No orphaned records were detected.
+3.The Kimball Star Schema maintains full referential integrity.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Business Interpretation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+1.Most transactions are legitimate.
+2.Fraud transactions represent a very small percentage of the dataset.
+3.Only a small subset of fraud cases was flagged by the legacy fraud detection system.
+4.This imbalance highlights the importance of machine learning models for fraud detection.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Validation Completed Successfully
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Overall Result : PASS
+The data warehouse passed all quality assurance checks.
+The dataset is ready for SQL Analytics,
+Machine Learning and Power BI reporting.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -85,6 +328,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="13.5"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -94,7 +345,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -102,11 +353,61 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -114,11 +415,324 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="25">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -129,6 +743,60 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1C547D3D-F06B-45FD-9F00-D23296F75748}" name="Table2" displayName="Table2" ref="A1:D10" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20" headerRowBorderDxfId="23" tableBorderDxfId="24" totalsRowBorderDxfId="22">
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{B39278FB-6462-4F5B-A044-3A71B39DB65A}" name="Validation Check" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{C3C5DD06-254B-45FC-B50A-076D3FF23057}" name="Expected Result" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{697D1D8D-1D9C-4002-81E9-F2C29556C44E}" name="Actual Result" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{7372E1FB-427E-4143-B7E9-6324BAEECC0B}" name="Status" dataDxfId="16"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F95F3BA4-08FF-494A-BC3C-9C41C6E689E8}" name="Table3" displayName="Table3" ref="A1:C4" totalsRowShown="0" headerRowDxfId="13">
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{32E96CE9-7790-44DE-94D5-014B6DCC3D5B}" name="IsFraud" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{BC22F00E-1579-4C0C-8ED5-C12D46F1AB0C}" name="IsFlaggedFraud" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{D63D298A-4160-4F71-88D3-D3695150DCC5}" name="Transactions"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F52F95BF-1923-4747-AA9E-1518DCEF627F}" name="Table4" displayName="Table4" ref="A1:C6" totalsRowShown="0" headerRowDxfId="8" dataDxfId="9">
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{BFD0BDCC-D132-4C23-8570-226A288DF076}" name="Dimension" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{0B7FCD1A-E370-41F1-8EB7-116C124871C1}" name="Orphan Records" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{FA0B634C-EF5D-4DC0-9743-939313793DFD}" name="Status" dataDxfId="10"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{06EA43A8-96EC-4A20-BDB7-1D832094B593}" name="Table5" displayName="Table5" ref="A1:B7" totalsRowShown="0" headerRowDxfId="4" dataDxfId="5">
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{4F8905AA-8F4F-4D91-BE15-DD30C4D9CC69}" name="Check" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{9553A557-F04A-4B02-B2AE-620DF628AA53}" name="Result" dataDxfId="6"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{80C2B841-08E5-4A98-A65B-A4AC61E49288}" name="Table6" displayName="Table6" ref="A3:B8" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{0D45A19E-BA96-4320-8851-55235C5B9847}" name="Metric" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{38031073-22CE-427D-8BB3-9B819FE9849C}" name="Value" dataDxfId="2"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -447,63 +1115,507 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CC40876-82A2-4021-9A53-700435E5B0D3}">
-  <dimension ref="A1:B6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D81C1064-605D-4057-81E4-902822EC5975}">
+  <dimension ref="A1:I15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.6640625" customWidth="1"/>
-    <col min="2" max="2" width="15.88671875" customWidth="1"/>
+    <col min="1" max="1" width="18.21875" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" style="4" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" customWidth="1"/>
+    <col min="8" max="8" width="8.88671875" customWidth="1"/>
+    <col min="9" max="9" width="56.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="9">
+        <v>6362620</v>
+      </c>
+      <c r="C2" s="9">
+        <v>6362620</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="10">
+        <v>0</v>
+      </c>
+      <c r="C3" s="10">
+        <v>0</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="10">
+        <v>0</v>
+      </c>
+      <c r="C4" s="10">
+        <v>0</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4" s="11"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="10">
+        <v>0</v>
+      </c>
+      <c r="C5" s="10">
+        <v>0</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="10">
+        <v>0</v>
+      </c>
+      <c r="C6" s="10">
+        <v>0</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="10">
+        <v>0</v>
+      </c>
+      <c r="C7" s="10">
+        <v>0</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="10">
+        <v>0</v>
+      </c>
+      <c r="C8" s="10">
+        <v>0</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="10">
+        <v>0</v>
+      </c>
+      <c r="C9" s="10">
+        <v>0</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="10">
+        <v>0</v>
+      </c>
+      <c r="C10" s="10">
+        <v>0</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="14"/>
+    </row>
+    <row r="15" spans="1:9" ht="216" x14ac:dyDescent="0.3">
+      <c r="A15" s="13"/>
+      <c r="B15" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" s="13"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B11B0AD2-BBF5-4A21-B1B3-1209FEEFEBB9}">
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.109375" customWidth="1"/>
+    <col min="2" max="2" width="27" customWidth="1"/>
+    <col min="3" max="3" width="11.109375" customWidth="1"/>
+    <col min="6" max="6" width="49.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2">
+        <v>0</v>
+      </c>
+      <c r="B2" s="16">
+        <v>0</v>
+      </c>
+      <c r="C2" s="15">
+        <v>6354407</v>
+      </c>
+      <c r="F2" s="11"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
         <v>1</v>
+      </c>
+      <c r="B3" s="2">
+        <v>0</v>
+      </c>
+      <c r="C3" s="3">
+        <v>8197</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="B7" s="12" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="12"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19C4F71E-B8D4-43C6-BDC1-D1FF47FC8B4B}">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.77734375" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="2">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="2">
+        <v>0</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="2">
+        <v>0</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="2">
+        <v>0</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="B10" s="12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{888075F8-1146-424A-A99A-1498A45FDA0F}">
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="21.77734375" customWidth="1"/>
+    <col min="2" max="2" width="22.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>3</v>
+        <v>27</v>
+      </c>
+      <c r="B2" s="2">
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+      <c r="B3" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>3</v>
+        <v>29</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+      <c r="B5" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>3</v>
+        <v>31</v>
+      </c>
+      <c r="B6" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="1:2" ht="175.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="12"/>
+      <c r="B10" s="12" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6DB642E-70D1-4016-AC64-88C17103B24C}">
+  <dimension ref="A1:O11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="12.109375" customWidth="1"/>
+    <col min="6" max="6" width="5" customWidth="1"/>
+    <col min="7" max="15" width="8.88671875" hidden="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" ht="18" x14ac:dyDescent="0.3">
+      <c r="A1" s="17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="3">
+        <v>6362620</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="89.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" s="18"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="18"/>
+      <c r="J11" s="18"/>
+      <c r="K11" s="18"/>
+      <c r="L11" s="18"/>
+      <c r="M11" s="18"/>
+      <c r="N11" s="18"/>
+      <c r="O11" s="18"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A11:O11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>